<commit_message>
correction slicing participants 6697746d343b4d66138c6f1149dd33ed58d47e36
</commit_message>
<xml_diff>
--- a/fix/slicing-type-this/ig/StructureDefinition-fr-cda-participant-corps.xlsx
+++ b/fix/slicing-type-this/ig/StructureDefinition-fr-cda-participant-corps.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AK$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AK$35</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="186">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-07T09:51:04+00:00</t>
+    <t>2026-10-08T08:06:17+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -408,6 +408,24 @@
     <t>InfrastructureRoot.templateId</t>
   </si>
   <si>
+    <t>Participant2.templateId.nullFlavor</t>
+  </si>
+  <si>
+    <t>Participant2.templateId.assigningAuthorityName</t>
+  </si>
+  <si>
+    <t>Participant2.templateId.displayable</t>
+  </si>
+  <si>
+    <t>Participant2.templateId.root</t>
+  </si>
+  <si>
+    <t>A unique identifier that guarantees the global uniqueness of the instance identifier. The root alone may be the entire instance identifier.</t>
+  </si>
+  <si>
+    <t>Participant2.templateId.extension</t>
+  </si>
+  <si>
     <t>Participant2.templateId:templateId</t>
   </si>
   <si>
@@ -420,70 +438,28 @@
     <t>Participant2.templateId:templateId.nullFlavor</t>
   </si>
   <si>
-    <t>Participant2.templateId.nullFlavor</t>
-  </si>
-  <si>
     <t>Participant2.templateId:templateId.assigningAuthorityName</t>
   </si>
   <si>
-    <t>Participant2.templateId.assigningAuthorityName</t>
-  </si>
-  <si>
     <t>Participant2.templateId:templateId.displayable</t>
   </si>
   <si>
-    <t>Participant2.templateId.displayable</t>
-  </si>
-  <si>
     <t>Participant2.templateId:templateId.root</t>
   </si>
   <si>
-    <t>Participant2.templateId.root</t>
-  </si>
-  <si>
-    <t>A unique identifier that guarantees the global uniqueness of the instance identifier. The root alone may be the entire instance identifier.</t>
-  </si>
-  <si>
     <t>1.2.250.1.213.1.1.3.109</t>
   </si>
   <si>
     <t>Participant2.templateId:templateId.extension</t>
   </si>
   <si>
-    <t>Participant2.templateId.extension</t>
-  </si>
-  <si>
-    <t>Participant2.templateId:templateId-other</t>
-  </si>
-  <si>
-    <t>templateId-other</t>
-  </si>
-  <si>
-    <t>Autre TemplateId</t>
-  </si>
-  <si>
-    <t>Participant2.templateId:templateId-other.nullFlavor</t>
-  </si>
-  <si>
-    <t>Participant2.templateId:templateId-other.assigningAuthorityName</t>
-  </si>
-  <si>
-    <t>Participant2.templateId:templateId-other.displayable</t>
-  </si>
-  <si>
-    <t>Participant2.templateId:templateId-other.root</t>
+    <t>Participant2.typeCode</t>
   </si>
   <si>
     <t>Y</t>
   </si>
   <si>
-    <t>Participant2.templateId:templateId-other.extension</t>
-  </si>
-  <si>
-    <t>Participant2.typeCode</t>
-  </si>
-  <si>
-    <t>http://hl7.org/cda/stds/core/ValueSet/CDAParticipationType|2.0.3-sd</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ParticipationType-cisis|20260916095457</t>
   </si>
   <si>
     <t>Participant2.contextControlCode</t>
@@ -930,12 +906,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK36"/>
+  <dimension ref="A1:AK35"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="53.1484375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="48.39453125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="39.30859375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="14.20703125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="21.37890625" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
@@ -958,7 +934,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="18.49609375" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="54.46484375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="73.28515625" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
@@ -2109,15 +2085,15 @@
         <v>127</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>121</v>
-      </c>
-      <c r="C12" t="s" s="2">
-        <v>128</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E12" s="2"/>
+      <c r="E12" t="s" s="2">
+        <v>85</v>
+      </c>
       <c r="F12" t="s" s="2">
         <v>81</v>
       </c>
@@ -2134,13 +2110,11 @@
         <v>75</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="L12" t="s" s="2">
-        <v>129</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="L12" s="2"/>
       <c r="M12" t="s" s="2">
-        <v>129</v>
+        <v>87</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2167,13 +2141,11 @@
         <v>75</v>
       </c>
       <c r="X12" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y12" t="s" s="2">
-        <v>75</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="Y12" s="2"/>
       <c r="Z12" t="s" s="2">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="AA12" t="s" s="2">
         <v>75</v>
@@ -2191,13 +2163,13 @@
         <v>75</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>126</v>
+        <v>90</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH12" t="s" s="2">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="AI12" t="s" s="2">
         <v>75</v>
@@ -2211,17 +2183,17 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E13" t="s" s="2">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="F13" t="s" s="2">
         <v>81</v>
@@ -2239,11 +2211,11 @@
         <v>75</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="L13" s="2"/>
       <c r="M13" t="s" s="2">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
@@ -2270,11 +2242,13 @@
         <v>75</v>
       </c>
       <c r="X13" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="Y13" s="2"/>
+        <v>75</v>
+      </c>
+      <c r="Y13" t="s" s="2">
+        <v>75</v>
+      </c>
       <c r="Z13" t="s" s="2">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="AA13" t="s" s="2">
         <v>75</v>
@@ -2292,7 +2266,7 @@
         <v>75</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>81</v>
@@ -2312,17 +2286,17 @@
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E14" t="s" s="2">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="F14" t="s" s="2">
         <v>81</v>
@@ -2340,11 +2314,11 @@
         <v>75</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="L14" s="2"/>
       <c r="M14" t="s" s="2">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2395,7 +2369,7 @@
         <v>75</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>81</v>
@@ -2415,20 +2389,20 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E15" t="s" s="2">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="F15" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="G15" t="s" s="2">
         <v>76</v>
@@ -2443,11 +2417,11 @@
         <v>75</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="L15" s="2"/>
       <c r="M15" t="s" s="2">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2498,7 +2472,7 @@
         <v>75</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>81</v>
@@ -2518,20 +2492,20 @@
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E16" t="s" s="2">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="F16" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G16" t="s" s="2">
         <v>76</v>
@@ -2546,11 +2520,11 @@
         <v>75</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" t="s" s="2">
-        <v>138</v>
+        <v>119</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -2562,7 +2536,7 @@
         <v>75</v>
       </c>
       <c r="S16" t="s" s="2">
-        <v>139</v>
+        <v>75</v>
       </c>
       <c r="T16" t="s" s="2">
         <v>75</v>
@@ -2601,7 +2575,7 @@
         <v>75</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>81</v>
@@ -2621,18 +2595,18 @@
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>141</v>
-      </c>
-      <c r="C17" s="2"/>
+        <v>121</v>
+      </c>
+      <c r="C17" t="s" s="2">
+        <v>134</v>
+      </c>
       <c r="D17" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E17" t="s" s="2">
-        <v>118</v>
-      </c>
+      <c r="E17" s="2"/>
       <c r="F17" t="s" s="2">
         <v>81</v>
       </c>
@@ -2649,11 +2623,13 @@
         <v>75</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="L17" s="2"/>
+        <v>96</v>
+      </c>
+      <c r="L17" t="s" s="2">
+        <v>135</v>
+      </c>
       <c r="M17" t="s" s="2">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2704,13 +2680,13 @@
         <v>75</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH17" t="s" s="2">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="AI17" t="s" s="2">
         <v>75</v>
@@ -2724,23 +2700,23 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>121</v>
-      </c>
-      <c r="C18" t="s" s="2">
-        <v>143</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E18" s="2"/>
+      <c r="E18" t="s" s="2">
+        <v>85</v>
+      </c>
       <c r="F18" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G18" t="s" s="2">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="H18" t="s" s="2">
         <v>75</v>
@@ -2752,13 +2728,11 @@
         <v>75</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="L18" t="s" s="2">
-        <v>144</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="L18" s="2"/>
       <c r="M18" t="s" s="2">
-        <v>144</v>
+        <v>87</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -2785,13 +2759,11 @@
         <v>75</v>
       </c>
       <c r="X18" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y18" t="s" s="2">
-        <v>75</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="Y18" s="2"/>
       <c r="Z18" t="s" s="2">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="AA18" t="s" s="2">
         <v>75</v>
@@ -2809,13 +2781,13 @@
         <v>75</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>126</v>
+        <v>90</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH18" t="s" s="2">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="AI18" t="s" s="2">
         <v>75</v>
@@ -2829,17 +2801,17 @@
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E19" t="s" s="2">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="F19" t="s" s="2">
         <v>81</v>
@@ -2857,11 +2829,11 @@
         <v>75</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" t="s" s="2">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2888,11 +2860,13 @@
         <v>75</v>
       </c>
       <c r="X19" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="Y19" s="2"/>
+        <v>75</v>
+      </c>
+      <c r="Y19" t="s" s="2">
+        <v>75</v>
+      </c>
       <c r="Z19" t="s" s="2">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>75</v>
@@ -2910,7 +2884,7 @@
         <v>75</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>81</v>
@@ -2930,17 +2904,17 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E20" t="s" s="2">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="F20" t="s" s="2">
         <v>81</v>
@@ -2958,11 +2932,11 @@
         <v>75</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" t="s" s="2">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -3013,7 +2987,7 @@
         <v>75</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>81</v>
@@ -3033,20 +3007,20 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E21" t="s" s="2">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="F21" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="G21" t="s" s="2">
         <v>76</v>
@@ -3061,11 +3035,11 @@
         <v>75</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" t="s" s="2">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -3077,7 +3051,7 @@
         <v>75</v>
       </c>
       <c r="S21" t="s" s="2">
-        <v>75</v>
+        <v>140</v>
       </c>
       <c r="T21" t="s" s="2">
         <v>75</v>
@@ -3116,7 +3090,7 @@
         <v>75</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>81</v>
@@ -3134,28 +3108,28 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E22" t="s" s="2">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="F22" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G22" t="s" s="2">
         <v>76</v>
       </c>
       <c r="H22" t="s" s="2">
-        <v>149</v>
+        <v>75</v>
       </c>
       <c r="I22" t="s" s="2">
         <v>75</v>
@@ -3164,11 +3138,11 @@
         <v>75</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="L22" s="2"/>
       <c r="M22" t="s" s="2">
-        <v>138</v>
+        <v>119</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3219,7 +3193,7 @@
         <v>75</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>81</v>
@@ -3237,28 +3211,26 @@
         <v>75</v>
       </c>
     </row>
-    <row r="23" hidden="true">
+    <row r="23">
       <c r="A23" t="s" s="2">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E23" t="s" s="2">
-        <v>118</v>
-      </c>
+      <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="G23" t="s" s="2">
         <v>76</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>75</v>
+        <v>143</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>75</v>
@@ -3267,12 +3239,10 @@
         <v>75</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="L23" s="2"/>
-      <c r="M23" t="s" s="2">
-        <v>119</v>
-      </c>
+      <c r="M23" s="2"/>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -3298,13 +3268,11 @@
         <v>75</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y23" t="s" s="2">
-        <v>75</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="Y23" s="2"/>
       <c r="Z23" t="s" s="2">
-        <v>75</v>
+        <v>144</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>75</v>
@@ -3322,10 +3290,10 @@
         <v>75</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>120</v>
+        <v>142</v>
       </c>
       <c r="AG23" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AH23" t="s" s="2">
         <v>76</v>
@@ -3340,12 +3308,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3353,13 +3321,13 @@
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G24" t="s" s="2">
         <v>76</v>
       </c>
       <c r="H24" t="s" s="2">
-        <v>149</v>
+        <v>75</v>
       </c>
       <c r="I24" t="s" s="2">
         <v>75</v>
@@ -3379,7 +3347,7 @@
       </c>
       <c r="Q24" s="2"/>
       <c r="R24" t="s" s="2">
-        <v>75</v>
+        <v>146</v>
       </c>
       <c r="S24" t="s" s="2">
         <v>75</v>
@@ -3401,7 +3369,7 @@
       </c>
       <c r="Y24" s="2"/>
       <c r="Z24" t="s" s="2">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>75</v>
@@ -3419,10 +3387,10 @@
         <v>75</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="AG24" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AH24" t="s" s="2">
         <v>76</v>
@@ -3439,10 +3407,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -3465,7 +3433,7 @@
         <v>75</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>86</v>
+        <v>149</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
@@ -3476,7 +3444,7 @@
       </c>
       <c r="Q25" s="2"/>
       <c r="R25" t="s" s="2">
-        <v>154</v>
+        <v>75</v>
       </c>
       <c r="S25" t="s" s="2">
         <v>75</v>
@@ -3494,11 +3462,13 @@
         <v>75</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="Y25" s="2"/>
+        <v>75</v>
+      </c>
+      <c r="Y25" t="s" s="2">
+        <v>75</v>
+      </c>
       <c r="Z25" t="s" s="2">
-        <v>155</v>
+        <v>75</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>75</v>
@@ -3516,7 +3486,7 @@
         <v>75</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>81</v>
@@ -3534,12 +3504,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="26" hidden="true">
+    <row r="26">
       <c r="A26" t="s" s="2">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -3553,7 +3523,7 @@
         <v>76</v>
       </c>
       <c r="H26" t="s" s="2">
-        <v>75</v>
+        <v>143</v>
       </c>
       <c r="I26" t="s" s="2">
         <v>75</v>
@@ -3562,10 +3532,14 @@
         <v>75</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>157</v>
-      </c>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
+        <v>151</v>
+      </c>
+      <c r="L26" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="M26" t="s" s="2">
+        <v>152</v>
+      </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
@@ -3615,7 +3589,7 @@
         <v>75</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>81</v>
@@ -3633,18 +3607,20 @@
         <v>75</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E27" s="2"/>
+      <c r="E27" t="s" s="2">
+        <v>85</v>
+      </c>
       <c r="F27" t="s" s="2">
         <v>81</v>
       </c>
@@ -3652,7 +3628,7 @@
         <v>76</v>
       </c>
       <c r="H27" t="s" s="2">
-        <v>149</v>
+        <v>75</v>
       </c>
       <c r="I27" t="s" s="2">
         <v>75</v>
@@ -3661,13 +3637,11 @@
         <v>75</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>159</v>
-      </c>
-      <c r="L27" t="s" s="2">
-        <v>160</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="L27" s="2"/>
       <c r="M27" t="s" s="2">
-        <v>160</v>
+        <v>87</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3694,13 +3668,11 @@
         <v>75</v>
       </c>
       <c r="X27" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y27" t="s" s="2">
-        <v>75</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="Y27" s="2"/>
       <c r="Z27" t="s" s="2">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="AA27" t="s" s="2">
         <v>75</v>
@@ -3718,7 +3690,7 @@
         <v>75</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>158</v>
+        <v>90</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>81</v>
@@ -3738,18 +3710,16 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E28" t="s" s="2">
-        <v>85</v>
-      </c>
+      <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
         <v>81</v>
       </c>
@@ -3766,11 +3736,11 @@
         <v>75</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>86</v>
+        <v>155</v>
       </c>
       <c r="L28" s="2"/>
       <c r="M28" t="s" s="2">
-        <v>87</v>
+        <v>156</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -3797,11 +3767,13 @@
         <v>75</v>
       </c>
       <c r="X28" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="Y28" s="2"/>
+        <v>75</v>
+      </c>
+      <c r="Y28" t="s" s="2">
+        <v>75</v>
+      </c>
       <c r="Z28" t="s" s="2">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="AA28" t="s" s="2">
         <v>75</v>
@@ -3819,7 +3791,7 @@
         <v>75</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>90</v>
+        <v>157</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>81</v>
@@ -3839,10 +3811,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -3865,16 +3837,16 @@
         <v>75</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>163</v>
+        <v>86</v>
       </c>
       <c r="L29" s="2"/>
       <c r="M29" t="s" s="2">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
-        <v>75</v>
+        <v>160</v>
       </c>
       <c r="Q29" s="2"/>
       <c r="R29" t="s" s="2">
@@ -3896,13 +3868,11 @@
         <v>75</v>
       </c>
       <c r="X29" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y29" t="s" s="2">
-        <v>75</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="Y29" s="2"/>
       <c r="Z29" t="s" s="2">
-        <v>75</v>
+        <v>161</v>
       </c>
       <c r="AA29" t="s" s="2">
         <v>75</v>
@@ -3920,7 +3890,7 @@
         <v>75</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>81</v>
@@ -3938,18 +3908,20 @@
         <v>75</v>
       </c>
     </row>
-    <row r="30" hidden="true">
+    <row r="30">
       <c r="A30" t="s" s="2">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E30" s="2"/>
+      <c r="E30" t="s" s="2">
+        <v>164</v>
+      </c>
       <c r="F30" t="s" s="2">
         <v>81</v>
       </c>
@@ -3957,7 +3929,7 @@
         <v>76</v>
       </c>
       <c r="H30" t="s" s="2">
-        <v>75</v>
+        <v>143</v>
       </c>
       <c r="I30" t="s" s="2">
         <v>75</v>
@@ -3966,16 +3938,16 @@
         <v>75</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>86</v>
+        <v>165</v>
       </c>
       <c r="L30" s="2"/>
       <c r="M30" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
-        <v>168</v>
+        <v>75</v>
       </c>
       <c r="Q30" s="2"/>
       <c r="R30" t="s" s="2">
@@ -3997,11 +3969,13 @@
         <v>75</v>
       </c>
       <c r="X30" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="Y30" s="2"/>
+        <v>75</v>
+      </c>
+      <c r="Y30" t="s" s="2">
+        <v>75</v>
+      </c>
       <c r="Z30" t="s" s="2">
-        <v>169</v>
+        <v>75</v>
       </c>
       <c r="AA30" t="s" s="2">
         <v>75</v>
@@ -4019,7 +3993,7 @@
         <v>75</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>81</v>
@@ -4037,19 +4011,19 @@
         <v>75</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E31" t="s" s="2">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="F31" t="s" s="2">
         <v>81</v>
@@ -4058,7 +4032,7 @@
         <v>76</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>149</v>
+        <v>75</v>
       </c>
       <c r="I31" t="s" s="2">
         <v>75</v>
@@ -4067,11 +4041,11 @@
         <v>75</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="L31" s="2"/>
       <c r="M31" t="s" s="2">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4122,7 +4096,7 @@
         <v>75</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>81</v>
@@ -4142,17 +4116,17 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E32" t="s" s="2">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F32" t="s" s="2">
         <v>81</v>
@@ -4170,11 +4144,11 @@
         <v>75</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="L32" s="2"/>
       <c r="M32" t="s" s="2">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4225,7 +4199,7 @@
         <v>75</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>81</v>
@@ -4243,19 +4217,19 @@
         <v>75</v>
       </c>
     </row>
-    <row r="33" hidden="true">
+    <row r="33">
       <c r="A33" t="s" s="2">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E33" t="s" s="2">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F33" t="s" s="2">
         <v>81</v>
@@ -4264,7 +4238,7 @@
         <v>76</v>
       </c>
       <c r="H33" t="s" s="2">
-        <v>75</v>
+        <v>143</v>
       </c>
       <c r="I33" t="s" s="2">
         <v>75</v>
@@ -4273,11 +4247,11 @@
         <v>75</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="L33" s="2"/>
       <c r="M33" t="s" s="2">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -4328,7 +4302,7 @@
         <v>75</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>81</v>
@@ -4346,20 +4320,18 @@
         <v>75</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="E34" t="s" s="2">
-        <v>187</v>
-      </c>
+      <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
         <v>81</v>
       </c>
@@ -4367,21 +4339,19 @@
         <v>76</v>
       </c>
       <c r="H34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="I34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="J34" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="K34" t="s" s="2">
         <v>149</v>
       </c>
-      <c r="I34" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J34" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K34" t="s" s="2">
-        <v>173</v>
-      </c>
       <c r="L34" s="2"/>
-      <c r="M34" t="s" s="2">
-        <v>188</v>
-      </c>
+      <c r="M34" s="2"/>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
@@ -4431,7 +4401,7 @@
         <v>75</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>81</v>
@@ -4449,12 +4419,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="35" hidden="true">
+    <row r="35">
       <c r="A35" t="s" s="2">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4462,13 +4432,13 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="G35" t="s" s="2">
         <v>76</v>
       </c>
       <c r="H35" t="s" s="2">
-        <v>75</v>
+        <v>143</v>
       </c>
       <c r="I35" t="s" s="2">
         <v>75</v>
@@ -4477,10 +4447,14 @@
         <v>75</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>157</v>
-      </c>
-      <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
+        <v>184</v>
+      </c>
+      <c r="L35" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="M35" t="s" s="2">
+        <v>185</v>
+      </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -4530,10 +4504,10 @@
         <v>75</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="AG35" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AH35" t="s" s="2">
         <v>76</v>
@@ -4548,111 +4522,8 @@
         <v>75</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="s" s="2">
-        <v>191</v>
-      </c>
-      <c r="B36" t="s" s="2">
-        <v>191</v>
-      </c>
-      <c r="C36" s="2"/>
-      <c r="D36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E36" s="2"/>
-      <c r="F36" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G36" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H36" t="s" s="2">
-        <v>149</v>
-      </c>
-      <c r="I36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K36" t="s" s="2">
-        <v>192</v>
-      </c>
-      <c r="L36" t="s" s="2">
-        <v>193</v>
-      </c>
-      <c r="M36" t="s" s="2">
-        <v>193</v>
-      </c>
-      <c r="N36" s="2"/>
-      <c r="O36" s="2"/>
-      <c r="P36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q36" s="2"/>
-      <c r="R36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF36" t="s" s="2">
-        <v>191</v>
-      </c>
-      <c r="AG36" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH36" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ36" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK36" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AK36">
+  <autoFilter ref="A1:AK35">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -4662,7 +4533,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI35">
+  <conditionalFormatting sqref="A2:AI34">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>